<commit_message>
Record UNV-NOV1 Catch That approval and Universal Novice batch proposal
Catch That approved with functional Type, Universal tag, Novice tier, and no-roll wording. Remaining 12 proposed as a batch; Conditioned Body needs a limit decision.
</commit_message>
<xml_diff>
--- a/review/abilities/workbooks/31_Novice_Abilities.xlsx
+++ b/review/abilities/workbooks/31_Novice_Abilities.xlsx
@@ -336,7 +336,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -1178,8 +1177,8 @@
   </sheetData>
   <mergeCells count="24">
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A17:D17"/>
     <mergeCell ref="B11:D11"/>
-    <mergeCell ref="A17:D17"/>
     <mergeCell ref="A35:D35"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="A38:D38"/>
@@ -6587,12 +6586,12 @@
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Universal / Reaction / Skill</t>
         </is>
       </c>
       <c r="G54" s="9" t="inlineStr">
@@ -6602,7 +6601,7 @@
       </c>
       <c r="H54" s="9" t="inlineStr">
         <is>
-          <t>None — no roll</t>
+          <t>None (no roll)</t>
         </is>
       </c>
       <c r="I54" s="9" t="inlineStr">
@@ -6660,8 +6659,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="T54" s="9" t="inlineStr"/>
-      <c r="U54" s="9" t="inlineStr"/>
+      <c r="T54" s="9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U54" s="9" t="inlineStr">
+        <is>
+          <t>UNV-NOV1; approved 2026-10-29.</t>
+        </is>
+      </c>
       <c r="V54" s="9" t="inlineStr">
         <is>
           <t>catch-that.md</t>
@@ -19945,12 +19952,12 @@
       </c>
       <c r="J54" s="9" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="K54" s="9" t="inlineStr">
         <is>
-          <t>No requirement; policy gap (F02).</t>
+          <t>No requirement; Universal (no discipline).</t>
         </is>
       </c>
     </row>
@@ -25284,80 +25291,336 @@
       </c>
     </row>
     <row r="5" ht="16.5" customHeight="1">
-      <c r="A5" s="7" t="inlineStr"/>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr"/>
-      <c r="I5" s="7" t="inlineStr"/>
-      <c r="J5" s="7" t="inlineStr"/>
-      <c r="K5" s="7" t="inlineStr"/>
-      <c r="L5" s="7" t="inlineStr"/>
-      <c r="M5" s="7" t="inlineStr"/>
-      <c r="N5" s="7" t="inlineStr"/>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>CHG-UNV-001</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>catch-that</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Catch That!</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>design/cards/catch-that.md</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Skill / Utility</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Taxonomy</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Functional Type plus Tags for the Universal Novice standard.</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M5" s="7" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O5" s="7" t="inlineStr"/>
-      <c r="P5" s="7" t="inlineStr"/>
-      <c r="Q5" s="7" t="inlineStr"/>
+      <c r="P5" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q5" s="7" t="inlineStr">
+        <is>
+          <t>UNV-NOV1; approved in conversation.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="16.5" customHeight="1">
-      <c r="A6" s="9" t="inlineStr"/>
-      <c r="B6" s="9" t="inlineStr"/>
-      <c r="C6" s="9" t="inlineStr"/>
-      <c r="D6" s="9" t="inlineStr"/>
-      <c r="E6" s="9" t="inlineStr"/>
-      <c r="F6" s="9" t="inlineStr"/>
-      <c r="G6" s="9" t="inlineStr"/>
-      <c r="H6" s="9" t="inlineStr"/>
-      <c r="I6" s="9" t="inlineStr"/>
-      <c r="J6" s="9" t="inlineStr"/>
-      <c r="K6" s="9" t="inlineStr"/>
-      <c r="L6" s="9" t="inlineStr"/>
-      <c r="M6" s="9" t="inlineStr"/>
-      <c r="N6" s="9" t="inlineStr"/>
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>CHG-UNV-002</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>catch-that</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Catch That!</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>design/cards/catch-that.md</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>Universal / Reaction / Skill</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>Taxonomy</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>Marks the no-discipline category and the Reaction/Skill tags.</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N6" s="9" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O6" s="9" t="inlineStr"/>
-      <c r="P6" s="9" t="inlineStr"/>
-      <c r="Q6" s="9" t="inlineStr"/>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
+          <t>UNV-NOV1; approved in conversation.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="16.5" customHeight="1">
-      <c r="A7" s="7" t="inlineStr"/>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr"/>
-      <c r="I7" s="7" t="inlineStr"/>
-      <c r="J7" s="7" t="inlineStr"/>
-      <c r="K7" s="7" t="inlineStr"/>
-      <c r="L7" s="7" t="inlineStr"/>
-      <c r="M7" s="7" t="inlineStr"/>
-      <c r="N7" s="7" t="inlineStr"/>
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>CHG-UNV-003</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>catch-that</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Catch That!</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>design/cards/catch-that.md</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>None — no roll</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>None (no roll)</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>Removes the em dash and keeps the no-roll instruction.</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O7" s="7" t="inlineStr"/>
-      <c r="P7" s="7" t="inlineStr"/>
-      <c r="Q7" s="7" t="inlineStr"/>
+      <c r="P7" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q7" s="7" t="inlineStr">
+        <is>
+          <t>UNV-NOV1; approved in conversation.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="16.5" customHeight="1">
-      <c r="A8" s="9" t="inlineStr"/>
-      <c r="B8" s="9" t="inlineStr"/>
-      <c r="C8" s="9" t="inlineStr"/>
-      <c r="D8" s="9" t="inlineStr"/>
-      <c r="E8" s="9" t="inlineStr"/>
-      <c r="F8" s="9" t="inlineStr"/>
-      <c r="G8" s="9" t="inlineStr"/>
-      <c r="H8" s="9" t="inlineStr"/>
-      <c r="I8" s="9" t="inlineStr"/>
-      <c r="J8" s="9" t="inlineStr"/>
-      <c r="K8" s="9" t="inlineStr"/>
-      <c r="L8" s="9" t="inlineStr"/>
-      <c r="M8" s="9" t="inlineStr"/>
-      <c r="N8" s="9" t="inlineStr"/>
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>CHG-UNV-004</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>catch-that</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Catch That!</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>design/cards/catch-that.md</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Tier / minimum level</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Tier / minimum level: 1</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Tier: Novice · Minimum level: 1</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>Uses the agreed tier and minimum-level nomenclature.</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M8" s="9" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N8" s="9" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O8" s="9" t="inlineStr"/>
-      <c r="P8" s="9" t="inlineStr"/>
-      <c r="Q8" s="9" t="inlineStr"/>
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q8" s="9" t="inlineStr">
+        <is>
+          <t>UNV-NOV1; approved in conversation.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="16.5" customHeight="1">
       <c r="A9" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
Approve Universal Novice U1-U11 and record task-progress texts
Records CHG-UNV-005 through CHG-UNV-025. Carry the Wounded and Read the Room retain their stable IDs. Keep Your Bearings and Tell a Worthy Story use navigation and manipulation task progress; Read the Room uses investigation task progress.

A Party Piece uses the existing Musical Instrument item. Hold a Conversation and Conditioned Body remain pending; book cards are unchanged.
</commit_message>
<xml_diff>
--- a/review/abilities/workbooks/31_Novice_Abilities.xlsx
+++ b/review/abilities/workbooks/31_Novice_Abilities.xlsx
@@ -6260,19 +6260,17 @@
           <t>Level 1</t>
         </is>
       </c>
-      <c r="D51" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="D51" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Universal / Skill / Social / Passive</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
@@ -6282,17 +6280,17 @@
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>None — no roll</t>
+          <t>None (no roll)</t>
         </is>
       </c>
       <c r="I51" s="7" t="inlineStr">
         <is>
-          <t>Your own performance using the specialty chosen when you learn this ability.</t>
+          <t>Self, while playing your chosen instrument.</t>
         </is>
       </c>
       <c r="J51" s="7" t="inlineStr">
         <is>
-          <t>While performing the chosen specialty.</t>
+          <t>While you play the chosen instrument.</t>
         </is>
       </c>
       <c r="K51" s="7" t="inlineStr">
@@ -6302,17 +6300,21 @@
       </c>
       <c r="L51" s="7" t="inlineStr">
         <is>
-          <t>Purchase once; choose one specialty when learned.</t>
+          <t>Purchase once; choose one instrument when learned.</t>
         </is>
       </c>
       <c r="M51" s="7" t="inlineStr">
         <is>
-          <t>Gain a Boon to entertain through one specialty; 1 DP.</t>
+          <t>1 Boon to any Guile roll while playing your chosen instrument.</t>
         </is>
       </c>
       <c r="N51" s="7" t="inlineStr">
         <is>
-          <t>Choose one mundane performance specialty when you learn this ability, such as singing, juggling, storytelling or playing a particular instrument. Gain 1 Boon to Guile rolls made to entertain through that specialty. Use the ordinary task’s stakes and outcomes; this grants no automatic persuasion, deception or change of attitude. Anyone can attempt a performance without this ability, and a performance with no uncertain consequence needs no roll.</t>
+          <t>Action: Passive · Attribute: None (no roll)
+Target / range / shape: Self, while playing your chosen instrument.
+When you learn this ability, choose one ordinary instrument you own, such as a lute, flute, drum, fiddle or horn. While you play that instrument, gain 1 Boon to any Guile roll. The instrument must be in your hands and in playing condition. The Boon can support performance, persuasion, deception and other Guile approaches that the music carries. Ordinary performance remains available to everyone; a performance with no uncertain consequence needs no roll.
+Duration: While you play the chosen instrument.
+Equipment / acquisition: Requires an ordinary Musical Instrument (Bulk 1), chosen when you learn this ability; grants none.</t>
         </is>
       </c>
       <c r="O51" s="7" t="inlineStr">
@@ -6340,8 +6342,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="T51" s="7" t="inlineStr"/>
-      <c r="U51" s="7" t="inlineStr"/>
+      <c r="T51" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U51" s="7" t="inlineStr">
+        <is>
+          <t>UNV-NOV4; approved 2026-10-29.</t>
+        </is>
+      </c>
       <c r="V51" s="7" t="inlineStr">
         <is>
           <t>a-party-piece.md</t>
@@ -6364,19 +6374,17 @@
           <t>Level 1</t>
         </is>
       </c>
-      <c r="D52" s="9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="D52" s="9" t="n">
+        <v>1</v>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Universal / Skill / Passive</t>
         </is>
       </c>
       <c r="G52" s="9" t="inlineStr">
@@ -6386,7 +6394,7 @@
       </c>
       <c r="H52" s="9" t="inlineStr">
         <is>
-          <t>None — no roll</t>
+          <t>None (no roll)</t>
         </is>
       </c>
       <c r="I52" s="9" t="inlineStr">
@@ -6411,12 +6419,16 @@
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>Learn one ordinary language; 1 DP.</t>
+          <t>Choose one ordinary language; speak, understand, read and write it.</t>
         </is>
       </c>
       <c r="N52" s="9" t="inlineStr">
         <is>
-          <t>When you learn this ability, choose one ordinary language you do not already know. You can speak and understand it, and read and write its usual script if it has one. Record the language on your sheet. A signed language uses signing instead of speech. Choose from the campaign’s ordinary languages with the DA; this grants no secret or supernatural language.</t>
+          <t>Action: Passive · Attribute: None (no roll)
+Target / range / shape: Self
+When you learn this ability, choose one ordinary language you do not already know. You can speak and understand it, and read and write its usual script if it has one. Record the language on your sheet. A signed language uses signing instead of speech. Choose from the campaign's ordinary languages with the DA. Secret and supernatural languages are learned through their own paths.
+Duration: Permanent knowledge of the chosen language.
+Equipment / acquisition: None.</t>
         </is>
       </c>
       <c r="O52" s="9" t="inlineStr">
@@ -6444,8 +6456,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="T52" s="9" t="inlineStr"/>
-      <c r="U52" s="9" t="inlineStr"/>
+      <c r="T52" s="9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U52" s="9" t="inlineStr">
+        <is>
+          <t>UNV-NOV2; approved 2026-10-29.</t>
+        </is>
+      </c>
       <c r="V52" s="9" t="inlineStr">
         <is>
           <t>another-tongue.md</t>
@@ -6455,7 +6475,7 @@
     <row r="53" ht="129" customHeight="1">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>Catch a Falling Friend</t>
+          <t>Carry the Wounded</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -6468,24 +6488,22 @@
           <t>Level 1</t>
         </is>
       </c>
-      <c r="D53" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="D53" s="7" t="n">
+        <v>2</v>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Movement</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Universal / Skill / Support</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>Reaction</t>
+          <t>Maneuver</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr">
@@ -6495,12 +6513,12 @@
       </c>
       <c r="I53" s="7" t="inlineStr">
         <is>
-          <t>One adjacent willing creature beginning to fall</t>
+          <t>One adjacent willing creature, or one adjacent creature at 0 HP.</t>
         </is>
       </c>
       <c r="J53" s="7" t="inlineStr">
         <is>
-          <t>Resolve once at the stated trigger; applied conditions follow normal decay.</t>
+          <t>While you carry them.</t>
         </is>
       </c>
       <c r="K53" s="7" t="inlineStr">
@@ -6515,17 +6533,16 @@
       </c>
       <c r="M53" s="7" t="inlineStr">
         <is>
-          <t>Catch a falling companion at an edge.</t>
+          <t>Carry an adjacent willing or 0 HP creature at half Speed.</t>
         </is>
       </c>
       <c r="N53" s="7" t="inlineStr">
         <is>
-          <t>Reaction; requires a free hand and secure footing at the start. Weak and Standard leave the friend held at the edge until moved or released. If no support could bear both, DA states that before use; no impossible attempt.
-• Weak: Stop its fall; you drop prone at the edge.
-• Standard: Stop its fall and keep your footing.
-• Strong: Stop its fall and pull it into an adjacent free safe square.
-Stability exception: this willing rescue movement ignores Stability.
-It does not allow moving an unwilling target or bypassing a grapple.</t>
+          <t>Action: Maneuver · Attribute: Brawn
+Target / range / shape: One adjacent willing creature, or one adjacent creature at 0 HP.
+You can move with the creature at half your Speed. The creature moves with you and ends adjacent. You can carry them through doors, up stairs and across ordinary terrain. If you fall prone, you set them down safely in an adjacent square. One creature at a time; a second carrier or a litter can share the load.
+Duration: While you carry them.
+Equipment / acquisition: Requires a free hand; grants none.</t>
         </is>
       </c>
       <c r="O53" s="7" t="inlineStr">
@@ -6555,8 +6572,16 @@
 Move it into Rules.</t>
         </is>
       </c>
-      <c r="T53" s="7" t="inlineStr"/>
-      <c r="U53" s="7" t="inlineStr"/>
+      <c r="T53" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U53" s="7" t="inlineStr">
+        <is>
+          <t>UNV-NOV7; approved 2026-10-29.</t>
+        </is>
+      </c>
       <c r="V53" s="7" t="inlineStr">
         <is>
           <t>catch-a-falling-friend.md</t>
@@ -6579,10 +6604,8 @@
           <t>Level 1</t>
         </is>
       </c>
-      <c r="D54" s="9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="D54" s="9" t="n">
+        <v>1</v>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
@@ -6606,7 +6629,7 @@
       </c>
       <c r="I54" s="9" t="inlineStr">
         <is>
-          <t>One falling, unattended item in your square or an adjacent square, within reach. Before it lands or falls out of reach.</t>
+          <t>One falling, unattended item in your square or an adjacent square, within reach, before it lands or falls out of reach.</t>
         </is>
       </c>
       <c r="J54" s="9" t="inlineStr">
@@ -6626,12 +6649,16 @@
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>Catch a falling item in a free hand; 1 DP.</t>
+          <t>Catch a small falling unattended item in a free hand.</t>
         </is>
       </c>
       <c r="N54" s="9" t="inlineStr">
         <is>
-          <t>Catch the item in a free hand. It must be small enough to hold in that hand. This cannot intercept an attack or take an item another creature is holding.</t>
+          <t>Action: Reaction · Attribute: None (no roll)
+Target / range / shape: One falling, unattended item in your square or an adjacent square, within reach, before it lands or falls out of reach.
+Catch the item in a free hand. The item must be small enough to hold in that hand. The ability catches falling objects; attacks and items held by another creature follow their own rules.
+Duration: Instant.
+Equipment / acquisition: None.</t>
         </is>
       </c>
       <c r="O54" s="9" t="inlineStr">
@@ -6666,7 +6693,7 @@
       </c>
       <c r="U54" s="9" t="inlineStr">
         <is>
-          <t>UNV-NOV1; approved 2026-10-29.</t>
+          <t>UNV-NOV1; approved 2026-10-29. Positive wording cleanup.</t>
         </is>
       </c>
       <c r="V54" s="9" t="inlineStr">
@@ -6904,19 +6931,17 @@
           <t>Level 1</t>
         </is>
       </c>
-      <c r="D57" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="D57" s="7" t="n">
+        <v>2</v>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Universal / Skill / Exploration</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
@@ -6931,12 +6956,12 @@
       </c>
       <c r="I57" s="7" t="inlineStr">
         <is>
-          <t>An unfamiliar place with usable landmarks; one minute</t>
+          <t>A navigation task in an unfamiliar place with usable landmarks.</t>
         </is>
       </c>
       <c r="J57" s="7" t="inlineStr">
         <is>
-          <t>Information and earned progress persist for the stated task; completed changes remain until circumstances alter them.</t>
+          <t>The progress persists for the navigation task.</t>
         </is>
       </c>
       <c r="K57" s="7" t="inlineStr">
@@ -6951,15 +6976,20 @@
       </c>
       <c r="M57" s="7" t="inlineStr">
         <is>
-          <t>Navigate with landmarks and clear bearings.</t>
+          <t>Make a navigation check for 1/2/3 progress.</t>
         </is>
       </c>
       <c r="N57" s="7" t="inlineStr">
         <is>
-          <t>Ordinary navigation is possible without the card. No routine travel roll; only consequential uncertainty. No magic compass when evidence is absent.
-• Weak: 1 progress toward finding your way; identify a visible landmark you can use to retrace this attempt.
-• Standard: 2 progress and identify your return direction.
-• Strong: 3 progress and describe a recognizable landmark to companions.</t>
+          <t>Action: Main Action · Attribute: Reason
+Time: One minute per attempt.
+Target / range / shape: A navigation task in an unfamiliar place with usable landmarks.
+Make a navigation check to make progress toward the navigation task.
+• Weak: 1 progress.
+• Standard: 2 progress.
+• Strong: 3 progress.
+Duration: The progress persists for the navigation task.
+Equipment / acquisition: None.</t>
         </is>
       </c>
       <c r="O57" s="7" t="inlineStr">
@@ -6987,8 +7017,16 @@
           <t>Assign a discipline requirement or formalize a General category.</t>
         </is>
       </c>
-      <c r="T57" s="7" t="inlineStr"/>
-      <c r="U57" s="7" t="inlineStr"/>
+      <c r="T57" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U57" s="7" t="inlineStr">
+        <is>
+          <t>UNV-NOV8; approved 2026-10-29.</t>
+        </is>
+      </c>
       <c r="V57" s="7" t="inlineStr">
         <is>
           <t>keep-your-bearings.md</t>
@@ -7011,19 +7049,17 @@
           <t>Level 1</t>
         </is>
       </c>
-      <c r="D58" s="9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="D58" s="9" t="n">
+        <v>1</v>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Skill / Defense</t>
+          <t>Defense</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Universal / Skill / Reaction</t>
         </is>
       </c>
       <c r="G58" s="9" t="inlineStr">
@@ -7033,7 +7069,7 @@
       </c>
       <c r="H58" s="9" t="inlineStr">
         <is>
-          <t>None — no roll</t>
+          <t>None (no roll)</t>
         </is>
       </c>
       <c r="I58" s="9" t="inlineStr">
@@ -7058,12 +7094,16 @@
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>Give an ally a defense Boon against an adjacent attacker; 1 DP.</t>
+          <t>Grant an ally 1 Boon to a sight-dependent defense roll.</t>
         </is>
       </c>
       <c r="N58" s="9" t="inlineStr">
         <is>
-          <t>Grant the ally 1 Boon to that defense roll. This momentary distraction does not create cover, make anyone Hidden or cancel the attack. Apply the normal Boon/Bane rules.</t>
+          <t>Action: Reaction · Attribute: None (no roll)
+Target / range / shape: One ally about to make a defense roll against a sight-dependent attack declared by an adjacent enemy that can see you. Before the roll.
+Grant the ally 1 Boon to that defense roll. The distraction affects the defense roll; the attack resolves normally. Apply the normal Boon/Bane rules.
+Duration: The triggering defense roll.
+Equipment / acquisition: None.</t>
         </is>
       </c>
       <c r="O58" s="9" t="inlineStr">
@@ -7091,8 +7131,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="T58" s="9" t="inlineStr"/>
-      <c r="U58" s="9" t="inlineStr"/>
+      <c r="T58" s="9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U58" s="9" t="inlineStr">
+        <is>
+          <t>UNV-NOV6; approved 2026-10-29.</t>
+        </is>
+      </c>
       <c r="V58" s="9" t="inlineStr">
         <is>
           <t>look-over-here.md</t>
@@ -7115,19 +7163,17 @@
           <t>Level 1</t>
         </is>
       </c>
-      <c r="D59" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="D59" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Universal / Skill</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
@@ -7137,7 +7183,7 @@
       </c>
       <c r="H59" s="7" t="inlineStr">
         <is>
-          <t>None — no roll</t>
+          <t>None (no roll)</t>
         </is>
       </c>
       <c r="I59" s="7" t="inlineStr">
@@ -7162,12 +7208,17 @@
       </c>
       <c r="M59" s="7" t="inlineStr">
         <is>
-          <t>Memorize one message of up to 50 words; 1 DP.</t>
+          <t>Memorize one message of up to 50 words exactly.</t>
         </is>
       </c>
       <c r="N59" s="7" t="inlineStr">
         <is>
-          <t>After rehearsing the message for one minute, you can reproduce its words exactly from memory. You may retain unfamiliar words this way without understanding them. You can retain only one message with this ability; memorizing another replaces it. Recalling the stored message requires only the normal time to speak or write it, not another minute of rehearsal. This grants no translation or additional ability.</t>
+          <t>Action: Main Action · Attribute: None (no roll)
+Time: One minute of rehearsal.
+Target / range / shape: One message of up to 50 words that you can hear, or read in a script you know.
+After rehearsing the message for one minute, you can reproduce its words exactly from memory. You may retain unfamiliar words this way without understanding them. You can retain one message at a time; memorizing another replaces it. Recalling the stored message takes only the normal time to speak or write it. Translation and understanding come from your own knowledge or other abilities.
+Duration: Until you memorize a replacement message.
+Equipment / acquisition: None.</t>
         </is>
       </c>
       <c r="O59" s="7" t="inlineStr">
@@ -7195,8 +7246,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="T59" s="7" t="inlineStr"/>
-      <c r="U59" s="7" t="inlineStr"/>
+      <c r="T59" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U59" s="7" t="inlineStr">
+        <is>
+          <t>UNV-NOV3; approved 2026-10-29.</t>
+        </is>
+      </c>
       <c r="V59" s="7" t="inlineStr">
         <is>
           <t>message-by-heart.md</t>
@@ -7206,7 +7265,7 @@
     <row r="60" ht="91.5" customHeight="1">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>Notice the Human Detail</t>
+          <t>Read the Room</t>
         </is>
       </c>
       <c r="B60" s="9" t="inlineStr">
@@ -7219,19 +7278,17 @@
           <t>Level 1</t>
         </is>
       </c>
-      <c r="D60" s="9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="D60" s="9" t="n">
+        <v>2</v>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Universal / Skill / Social / Investigation</t>
         </is>
       </c>
       <c r="G60" s="9" t="inlineStr">
@@ -7246,12 +7303,12 @@
       </c>
       <c r="I60" s="9" t="inlineStr">
         <is>
-          <t>An accessible scene or person you can examine; one minute</t>
+          <t>An investigation task about a social gathering or group you can observe.</t>
         </is>
       </c>
       <c r="J60" s="9" t="inlineStr">
         <is>
-          <t>Information and earned progress persist for the stated task; completed changes remain until circumstances alter them.</t>
+          <t>The progress persists for the investigation task.</t>
         </is>
       </c>
       <c r="K60" s="9" t="inlineStr">
@@ -7266,15 +7323,20 @@
       </c>
       <c r="M60" s="9" t="inlineStr">
         <is>
-          <t>Read visible clues and test an interpretation.</t>
+          <t>Make an investigation check for 1/2/3 progress.</t>
         </is>
       </c>
       <c r="N60" s="9" t="inlineStr">
         <is>
-          <t>No secret fact is invented. Obvious clues require no roll. This grants no lie detection, mind reading or an Observation attribute.
-• Weak: Learn one visible detail relevant to your stated question.
-• Standard: Also identify a plausible interpretation.
-• Strong: Also identify a concrete way to check that interpretation.</t>
+          <t>Action: Main Action · Attribute: Reason
+Time: One minute.
+Target / range / shape: An investigation task about a social gathering or group you can observe.
+Make an investigation check to make progress toward the investigation task.
+• Weak: 1 progress.
+• Standard: 2 progress.
+• Strong: 3 progress.
+Duration: The progress persists for the investigation task.
+Equipment / acquisition: None.</t>
         </is>
       </c>
       <c r="O60" s="9" t="inlineStr">
@@ -7302,8 +7364,16 @@
           <t>Assign a discipline requirement or formalize a General category.</t>
         </is>
       </c>
-      <c r="T60" s="9" t="inlineStr"/>
-      <c r="U60" s="9" t="inlineStr"/>
+      <c r="T60" s="9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U60" s="9" t="inlineStr">
+        <is>
+          <t>UNV-NOV9; approved 2026-10-29.</t>
+        </is>
+      </c>
       <c r="V60" s="9" t="inlineStr">
         <is>
           <t>notice-the-human-detail.md</t>
@@ -7326,19 +7396,17 @@
           <t>Level 1</t>
         </is>
       </c>
-      <c r="D61" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="D61" s="7" t="n">
+        <v>2</v>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Universal / Skill / Passive</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
@@ -7348,12 +7416,12 @@
       </c>
       <c r="H61" s="7" t="inlineStr">
         <is>
-          <t>None — no roll</t>
+          <t>None (no roll)</t>
         </is>
       </c>
       <c r="I61" s="7" t="inlineStr">
         <is>
-          <t>Your own carried inventory</t>
+          <t>Your own carried inventory.</t>
         </is>
       </c>
       <c r="J61" s="7" t="inlineStr">
@@ -7373,12 +7441,16 @@
       </c>
       <c r="M61" s="7" t="inlineStr">
         <is>
-          <t>Stow an item while drawing for an attack.</t>
+          <t>Once per turn, stow an item as part of drawing a different weapon.</t>
         </is>
       </c>
       <c r="N61" s="7" t="inlineStr">
         <is>
-          <t>Passive: once on your turn, stow one held ordinary item as part of drawing a different stowed weapon for an attack. The weapon still needs the required hands. Grants no free potion use, extra inventory slot or reduced Bulk.</t>
+          <t>Action: Passive · Attribute: None (no roll)
+Target / range / shape: Your own carried inventory.
+Once on your turn, stow one held ordinary item as part of drawing a different stowed weapon for an attack. The weapon still needs the required hands. The benefit covers the stow-and-draw; potions, inventory space and Bulk follow their normal rules.
+Duration: Once on each of your turns, when the printed weapon-switch trigger occurs.
+Equipment / acquisition: None.</t>
         </is>
       </c>
       <c r="O61" s="7" t="inlineStr">
@@ -7406,8 +7478,16 @@
           <t>Assign a discipline requirement or formalize a General category.</t>
         </is>
       </c>
-      <c r="T61" s="7" t="inlineStr"/>
-      <c r="U61" s="7" t="inlineStr"/>
+      <c r="T61" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U61" s="7" t="inlineStr">
+        <is>
+          <t>UNV-NOV10; approved 2026-10-29.</t>
+        </is>
+      </c>
       <c r="V61" s="7" t="inlineStr">
         <is>
           <t>pack-with-purpose.md</t>
@@ -7430,19 +7510,17 @@
           <t>Level 1</t>
         </is>
       </c>
-      <c r="D62" s="9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="D62" s="9" t="n">
+        <v>1</v>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Skill / Movement</t>
+          <t>Movement</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Universal / Skill / Passive</t>
         </is>
       </c>
       <c r="G62" s="9" t="inlineStr">
@@ -7452,7 +7530,7 @@
       </c>
       <c r="H62" s="9" t="inlineStr">
         <is>
-          <t>None — no roll</t>
+          <t>None (no roll)</t>
         </is>
       </c>
       <c r="I62" s="9" t="inlineStr">
@@ -7477,12 +7555,16 @@
       </c>
       <c r="M62" s="9" t="inlineStr">
         <is>
-          <t>Gain one movement square when you Disengage; 1 DP.</t>
+          <t>When you Disengage, gain 1 additional square of movement.</t>
         </is>
       </c>
       <c r="N62" s="9" t="inlineStr">
         <is>
-          <t>Gain 1 additional square of available movement for this turn. Spend it using normal terrain costs and movement restrictions. This does not increase Speed or add movement to each allowance gained by converting actions. Disengage’s protection from opportunity attacks applies normally.</t>
+          <t>Action: Passive · Attribute: None (no roll)
+Target / range / shape: Self, when you use Disengage.
+Gain 1 additional square of available movement this turn. Spend it using normal terrain costs and movement restrictions. The bonus applies to the Disengage movement; your Speed and converted movement allowances stay unchanged. Disengage's protection from opportunity attacks applies normally.
+Duration: Until the end of this turn; unused movement expires.
+Equipment / acquisition: None.</t>
         </is>
       </c>
       <c r="O62" s="9" t="inlineStr">
@@ -7510,8 +7592,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="T62" s="9" t="inlineStr"/>
-      <c r="U62" s="9" t="inlineStr"/>
+      <c r="T62" s="9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U62" s="9" t="inlineStr">
+        <is>
+          <t>UNV-NOV5; approved 2026-10-29.</t>
+        </is>
+      </c>
       <c r="V62" s="9" t="inlineStr">
         <is>
           <t>quick-exit.md</t>
@@ -7534,19 +7624,17 @@
           <t>Level 1</t>
         </is>
       </c>
-      <c r="D63" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="D63" s="7" t="n">
+        <v>2</v>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Universal / Skill / Social</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -7561,12 +7649,12 @@
       </c>
       <c r="I63" s="7" t="inlineStr">
         <is>
-          <t>A willing audience; a few minutes</t>
+          <t>A manipulation task involving one listener or a small audience that can understand you.</t>
         </is>
       </c>
       <c r="J63" s="7" t="inlineStr">
         <is>
-          <t>Information and earned progress persist for the stated task; completed changes remain until circumstances alter them.</t>
+          <t>The progress persists for the manipulation task.</t>
         </is>
       </c>
       <c r="K63" s="7" t="inlineStr">
@@ -7581,15 +7669,20 @@
       </c>
       <c r="M63" s="7" t="inlineStr">
         <is>
-          <t>Engage listeners and win an introduction.</t>
+          <t>Make a manipulation check for 1/2/3 progress.</t>
         </is>
       </c>
       <c r="N63" s="7" t="inlineStr">
         <is>
-          <t>Ordinary conversation remains available. Choose a plausible objective before rolling; this does not compel belief or behavior.
-• Weak: 1 progress toward engaging them; recognize one part of the story that visibly interests a listener.
-• Standard: 2 progress, that interest, and a volunteered local detail.
-• Strong: 3 progress, both details above, and an introduction to a willing listener.</t>
+          <t>Action: Main Action · Attribute: Guile
+Time: A few minutes.
+Target / range / shape: A manipulation task involving one listener or a small audience that can understand you.
+Choose a claim you want the listener to accept: a lie, a cover story, a rumor, or a version of events that favors you. Make a manipulation check to make progress toward the manipulation task.
+• Weak: 1 progress.
+• Standard: 2 progress.
+• Strong: 3 progress.
+Duration: The progress persists for the manipulation task.
+Equipment / acquisition: None.</t>
         </is>
       </c>
       <c r="O63" s="7" t="inlineStr">
@@ -7617,8 +7710,16 @@
           <t>Assign a discipline requirement or formalize a General category.</t>
         </is>
       </c>
-      <c r="T63" s="7" t="inlineStr"/>
-      <c r="U63" s="7" t="inlineStr"/>
+      <c r="T63" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U63" s="7" t="inlineStr">
+        <is>
+          <t>UNV-NOV11; approved 2026-10-29.</t>
+        </is>
+      </c>
       <c r="V63" s="7" t="inlineStr">
         <is>
           <t>tell-a-worthy-story.md</t>
@@ -19817,12 +19918,12 @@
       </c>
       <c r="J51" s="7" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="K51" s="7" t="inlineStr">
         <is>
-          <t>No requirement; policy gap (F02).</t>
+          <t>No requirement; Universal (no discipline).</t>
         </is>
       </c>
     </row>
@@ -19862,19 +19963,19 @@
       </c>
       <c r="J52" s="9" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="K52" s="9" t="inlineStr">
         <is>
-          <t>No requirement; policy gap (F02).</t>
+          <t>No requirement; Universal (no discipline).</t>
         </is>
       </c>
     </row>
     <row r="53" ht="16.5" customHeight="1">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>Catch a Falling Friend</t>
+          <t>Carry the Wounded</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -19902,17 +20003,17 @@
       </c>
       <c r="I53" s="7" t="inlineStr">
         <is>
-          <t>Reaction</t>
+          <t>Maneuver</t>
         </is>
       </c>
       <c r="J53" s="7" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Movement</t>
         </is>
       </c>
       <c r="K53" s="7" t="inlineStr">
         <is>
-          <t>No requirement; policy gap (F02).</t>
+          <t>No requirement; Universal (no discipline).</t>
         </is>
       </c>
     </row>
@@ -20087,12 +20188,12 @@
       </c>
       <c r="J57" s="7" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="K57" s="7" t="inlineStr">
         <is>
-          <t>No requirement; policy gap (F02).</t>
+          <t>No requirement; Universal (no discipline).</t>
         </is>
       </c>
     </row>
@@ -20132,12 +20233,12 @@
       </c>
       <c r="J58" s="9" t="inlineStr">
         <is>
-          <t>Skill / Defense</t>
+          <t>Defense</t>
         </is>
       </c>
       <c r="K58" s="9" t="inlineStr">
         <is>
-          <t>No requirement; policy gap (F02).</t>
+          <t>No requirement; Universal (no discipline).</t>
         </is>
       </c>
     </row>
@@ -20177,19 +20278,19 @@
       </c>
       <c r="J59" s="7" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="K59" s="7" t="inlineStr">
         <is>
-          <t>No requirement; policy gap (F02).</t>
+          <t>No requirement; Universal (no discipline).</t>
         </is>
       </c>
     </row>
     <row r="60" ht="16.5" customHeight="1">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>Notice the Human Detail</t>
+          <t>Read the Room</t>
         </is>
       </c>
       <c r="B60" s="9" t="inlineStr">
@@ -20222,12 +20323,12 @@
       </c>
       <c r="J60" s="9" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="K60" s="9" t="inlineStr">
         <is>
-          <t>No requirement; policy gap (F02).</t>
+          <t>No requirement; Universal (no discipline).</t>
         </is>
       </c>
     </row>
@@ -20267,12 +20368,12 @@
       </c>
       <c r="J61" s="7" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="K61" s="7" t="inlineStr">
         <is>
-          <t>No requirement; policy gap (F02).</t>
+          <t>No requirement; Universal (no discipline).</t>
         </is>
       </c>
     </row>
@@ -20312,12 +20413,12 @@
       </c>
       <c r="J62" s="9" t="inlineStr">
         <is>
-          <t>Skill / Movement</t>
+          <t>Movement</t>
         </is>
       </c>
       <c r="K62" s="9" t="inlineStr">
         <is>
-          <t>No requirement; policy gap (F02).</t>
+          <t>No requirement; Universal (no discipline).</t>
         </is>
       </c>
     </row>
@@ -20357,12 +20458,12 @@
       </c>
       <c r="J63" s="7" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="K63" s="7" t="inlineStr">
         <is>
-          <t>No requirement; policy gap (F02).</t>
+          <t>No requirement; Universal (no discipline).</t>
         </is>
       </c>
     </row>
@@ -25166,7 +25267,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25623,156 +25724,1747 @@
       </c>
     </row>
     <row r="9" ht="16.5" customHeight="1">
-      <c r="A9" s="7" t="inlineStr"/>
-      <c r="B9" s="7" t="inlineStr"/>
-      <c r="C9" s="7" t="inlineStr"/>
-      <c r="D9" s="7" t="inlineStr"/>
-      <c r="E9" s="7" t="inlineStr"/>
-      <c r="F9" s="7" t="inlineStr"/>
-      <c r="G9" s="7" t="inlineStr"/>
-      <c r="H9" s="7" t="inlineStr"/>
-      <c r="I9" s="7" t="inlineStr"/>
-      <c r="J9" s="7" t="inlineStr"/>
-      <c r="K9" s="7" t="inlineStr"/>
-      <c r="L9" s="7" t="inlineStr"/>
-      <c r="M9" s="7" t="inlineStr"/>
-      <c r="N9" s="7" t="inlineStr"/>
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>CHG-UNV-005</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>catch-that</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Catch That!</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>catch-that.md</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Card text</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Current catch limit used cannot wording.</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Positive wording; attacks and held items follow their own rules.</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>Wording</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>Positive wording; no mechanic change.</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M9" s="7" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O9" s="7" t="inlineStr"/>
-      <c r="P9" s="7" t="inlineStr"/>
-      <c r="Q9" s="7" t="inlineStr"/>
+      <c r="P9" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q9" s="7" t="inlineStr">
+        <is>
+          <t>UNV-NOV1; approved 2026-10-29; positive wording cleanup.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="16.5" customHeight="1">
-      <c r="A10" s="9" t="inlineStr"/>
-      <c r="B10" s="9" t="inlineStr"/>
-      <c r="C10" s="9" t="inlineStr"/>
-      <c r="D10" s="9" t="inlineStr"/>
-      <c r="E10" s="9" t="inlineStr"/>
-      <c r="F10" s="9" t="inlineStr"/>
-      <c r="G10" s="9" t="inlineStr"/>
-      <c r="H10" s="9" t="inlineStr"/>
-      <c r="I10" s="9" t="inlineStr"/>
-      <c r="J10" s="9" t="inlineStr"/>
-      <c r="K10" s="9" t="inlineStr"/>
-      <c r="L10" s="9" t="inlineStr"/>
-      <c r="M10" s="9" t="inlineStr"/>
-      <c r="N10" s="9" t="inlineStr"/>
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>CHG-UNV-006</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>another-tongue</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Another Tongue</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>another-tongue.md</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Tier / Type / Tags / Attribute</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>Tier / minimum level: 1; Type: Skill / Utility; Tags: —; Attribute: None — no roll</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>Tier: Novice · Minimum level: 1; Type: Utility; Tags: Universal / Skill / Passive; Attribute: None (no roll)</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>Taxonomy</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>Universal Novice standard: functional Type, Universal tag, Novice tier.</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M10" s="9" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N10" s="9" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O10" s="9" t="inlineStr"/>
-      <c r="P10" s="9" t="inlineStr"/>
-      <c r="Q10" s="9" t="inlineStr"/>
+      <c r="P10" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
+          <t>UNV-NOV2; approved 2026-10-29.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="16.5" customHeight="1">
-      <c r="A11" s="7" t="inlineStr"/>
-      <c r="B11" s="7" t="inlineStr"/>
-      <c r="C11" s="7" t="inlineStr"/>
-      <c r="D11" s="7" t="inlineStr"/>
-      <c r="E11" s="7" t="inlineStr"/>
-      <c r="F11" s="7" t="inlineStr"/>
-      <c r="G11" s="7" t="inlineStr"/>
-      <c r="H11" s="7" t="inlineStr"/>
-      <c r="I11" s="7" t="inlineStr"/>
-      <c r="J11" s="7" t="inlineStr"/>
-      <c r="K11" s="7" t="inlineStr"/>
-      <c r="L11" s="7" t="inlineStr"/>
-      <c r="M11" s="7" t="inlineStr"/>
-      <c r="N11" s="7" t="inlineStr"/>
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>CHG-UNV-007</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>another-tongue</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Another Tongue</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>another-tongue.md</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Card text</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Current text said it grants no secret or supernatural language.</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Positive wording; secret and supernatural languages are learned through their own paths.</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>Wording</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>Wording for the Universal Novice baseline.</t>
+        </is>
+      </c>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M11" s="7" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N11" s="7" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O11" s="7" t="inlineStr"/>
-      <c r="P11" s="7" t="inlineStr"/>
-      <c r="Q11" s="7" t="inlineStr"/>
+      <c r="P11" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q11" s="7" t="inlineStr">
+        <is>
+          <t>UNV-NOV2; approved 2026-10-29.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="16.5" customHeight="1">
-      <c r="A12" s="9" t="inlineStr"/>
-      <c r="B12" s="9" t="inlineStr"/>
-      <c r="C12" s="9" t="inlineStr"/>
-      <c r="D12" s="9" t="inlineStr"/>
-      <c r="E12" s="9" t="inlineStr"/>
-      <c r="F12" s="9" t="inlineStr"/>
-      <c r="G12" s="9" t="inlineStr"/>
-      <c r="H12" s="9" t="inlineStr"/>
-      <c r="I12" s="9" t="inlineStr"/>
-      <c r="J12" s="9" t="inlineStr"/>
-      <c r="K12" s="9" t="inlineStr"/>
-      <c r="L12" s="9" t="inlineStr"/>
-      <c r="M12" s="9" t="inlineStr"/>
-      <c r="N12" s="9" t="inlineStr"/>
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>CHG-UNV-008</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>message-by-heart</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Message by Heart</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>message-by-heart.md</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Tier / Type / Tags / Attribute</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Tier / minimum level: 1; Type: Skill / Utility; Tags: —; Attribute: None — no roll</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Tier: Novice · Minimum level: 1; Type: Utility; Tags: Universal / Skill; Attribute: None (no roll)</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>Taxonomy</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>Universal Novice standard: functional Type, Universal tag, Novice tier.</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L12" s="9" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M12" s="9" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N12" s="9" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O12" s="9" t="inlineStr"/>
-      <c r="P12" s="9" t="inlineStr"/>
-      <c r="Q12" s="9" t="inlineStr"/>
+      <c r="P12" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q12" s="9" t="inlineStr">
+        <is>
+          <t>UNV-NOV3; approved 2026-10-29.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="16.5" customHeight="1">
-      <c r="A13" s="7" t="inlineStr"/>
-      <c r="B13" s="7" t="inlineStr"/>
-      <c r="C13" s="7" t="inlineStr"/>
-      <c r="D13" s="7" t="inlineStr"/>
-      <c r="E13" s="7" t="inlineStr"/>
-      <c r="F13" s="7" t="inlineStr"/>
-      <c r="G13" s="7" t="inlineStr"/>
-      <c r="H13" s="7" t="inlineStr"/>
-      <c r="I13" s="7" t="inlineStr"/>
-      <c r="J13" s="7" t="inlineStr"/>
-      <c r="K13" s="7" t="inlineStr"/>
-      <c r="L13" s="7" t="inlineStr"/>
-      <c r="M13" s="7" t="inlineStr"/>
-      <c r="N13" s="7" t="inlineStr"/>
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>CHG-UNV-009</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>message-by-heart</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Message by Heart</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>message-by-heart.md</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Card text</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Current text said it grants no translation.</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Positive wording; translation comes from your own knowledge or other abilities.</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>Wording</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>Wording for the Universal Novice baseline.</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L13" s="7" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N13" s="7" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O13" s="7" t="inlineStr"/>
-      <c r="P13" s="7" t="inlineStr"/>
-      <c r="Q13" s="7" t="inlineStr"/>
+      <c r="P13" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q13" s="7" t="inlineStr">
+        <is>
+          <t>UNV-NOV3; approved 2026-10-29.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="16.5" customHeight="1">
-      <c r="A14" s="9" t="inlineStr"/>
-      <c r="B14" s="9" t="inlineStr"/>
-      <c r="C14" s="9" t="inlineStr"/>
-      <c r="D14" s="9" t="inlineStr"/>
-      <c r="E14" s="9" t="inlineStr"/>
-      <c r="F14" s="9" t="inlineStr"/>
-      <c r="G14" s="9" t="inlineStr"/>
-      <c r="H14" s="9" t="inlineStr"/>
-      <c r="I14" s="9" t="inlineStr"/>
-      <c r="J14" s="9" t="inlineStr"/>
-      <c r="K14" s="9" t="inlineStr"/>
-      <c r="L14" s="9" t="inlineStr"/>
-      <c r="M14" s="9" t="inlineStr"/>
-      <c r="N14" s="9" t="inlineStr"/>
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>CHG-UNV-010</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>a-party-piece</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>A Party Piece</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>a-party-piece.md</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Tier / Type / Tags / Attribute</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Tier / minimum level: 1; Type: Skill / Utility; Tags: —; Attribute: None — no roll</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>Tier: Novice · Minimum level: 1; Type: Utility; Tags: Universal / Skill / Social / Passive; Attribute: None (no roll)</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>Taxonomy</t>
+        </is>
+      </c>
+      <c r="J14" s="9" t="inlineStr">
+        <is>
+          <t>Universal Novice standard: functional Type, Universal tag, Novice tier.</t>
+        </is>
+      </c>
+      <c r="K14" s="9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L14" s="9" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M14" s="9" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N14" s="9" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O14" s="9" t="inlineStr"/>
-      <c r="P14" s="9" t="inlineStr"/>
-      <c r="Q14" s="9" t="inlineStr"/>
+      <c r="P14" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q14" s="9" t="inlineStr">
+        <is>
+          <t>UNV-NOV4; approved 2026-10-29.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="16.5" customHeight="1">
-      <c r="A15" s="7" t="inlineStr"/>
-      <c r="B15" s="7" t="inlineStr"/>
-      <c r="C15" s="7" t="inlineStr"/>
-      <c r="D15" s="7" t="inlineStr"/>
-      <c r="E15" s="7" t="inlineStr"/>
-      <c r="F15" s="7" t="inlineStr"/>
-      <c r="G15" s="7" t="inlineStr"/>
-      <c r="H15" s="7" t="inlineStr"/>
-      <c r="I15" s="7" t="inlineStr"/>
-      <c r="J15" s="7" t="inlineStr"/>
-      <c r="K15" s="7" t="inlineStr"/>
-      <c r="L15" s="7" t="inlineStr"/>
-      <c r="M15" s="7" t="inlineStr"/>
-      <c r="N15" s="7" t="inlineStr"/>
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>CHG-UNV-011</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>a-party-piece</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>A Party Piece</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>a-party-piece.md</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>Card text</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Choose a performance specialty; 1 Boon to Guile to entertain.</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Choose an instrument; 1 Boon to any Guile roll while playing it; uses the existing Musical Instrument item.</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>Mechanics</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>Mechanics for the Universal Novice baseline.</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N15" s="7" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O15" s="7" t="inlineStr"/>
-      <c r="P15" s="7" t="inlineStr"/>
-      <c r="Q15" s="7" t="inlineStr"/>
+      <c r="P15" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q15" s="7" t="inlineStr">
+        <is>
+          <t>UNV-NOV4; approved 2026-10-29.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="16.5" customHeight="1">
-      <c r="A16" s="9" t="inlineStr"/>
-      <c r="B16" s="9" t="inlineStr"/>
-      <c r="C16" s="9" t="inlineStr"/>
-      <c r="D16" s="9" t="inlineStr"/>
-      <c r="E16" s="9" t="inlineStr"/>
-      <c r="F16" s="9" t="inlineStr"/>
-      <c r="G16" s="9" t="inlineStr"/>
-      <c r="H16" s="9" t="inlineStr"/>
-      <c r="I16" s="9" t="inlineStr"/>
-      <c r="J16" s="9" t="inlineStr"/>
-      <c r="K16" s="9" t="inlineStr"/>
-      <c r="L16" s="9" t="inlineStr"/>
-      <c r="M16" s="9" t="inlineStr"/>
-      <c r="N16" s="9" t="inlineStr"/>
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>CHG-UNV-012</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>quick-exit</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Quick Exit</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>quick-exit.md</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Tier / Type / Tags / Attribute</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>Tier / minimum level: 1; Type: Skill / Movement; Tags: —; Attribute: None — no roll</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>Tier: Novice · Minimum level: 1; Type: Movement; Tags: Universal / Skill / Passive; Attribute: None (no roll)</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>Taxonomy</t>
+        </is>
+      </c>
+      <c r="J16" s="9" t="inlineStr">
+        <is>
+          <t>Universal Novice standard: functional Type, Universal tag, Novice tier.</t>
+        </is>
+      </c>
+      <c r="K16" s="9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L16" s="9" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M16" s="9" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N16" s="9" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O16" s="9" t="inlineStr"/>
-      <c r="P16" s="9" t="inlineStr"/>
-      <c r="Q16" s="9" t="inlineStr"/>
+      <c r="P16" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q16" s="9" t="inlineStr">
+        <is>
+          <t>UNV-NOV5; approved 2026-10-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CHG-UNV-013</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>quick-exit</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Quick Exit</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>quick-exit.md</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Card text</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Current text said it does not increase Speed.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Positive wording; Speed and converted movement stay unchanged.</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Wording</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Wording for the Universal Novice baseline.</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>UNV-NOV5; approved 2026-10-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CHG-UNV-014</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>look-over-here</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Look Over Here!</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>look-over-here.md</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Tier / Type / Tags / Attribute</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Tier / minimum level: 1; Type: Skill / Defense; Tags: —; Attribute: None — no roll</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Tier: Novice · Minimum level: 1; Type: Defense; Tags: Universal / Skill / Reaction; Attribute: None (no roll)</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Taxonomy</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Universal Novice standard: functional Type, Universal tag, Novice tier.</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>UNV-NOV6; approved 2026-10-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CHG-UNV-015</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>look-over-here</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Look Over Here!</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>look-over-here.md</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Card text</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Current text said it does not create cover.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Positive wording; the distraction affects the defense roll and the attack resolves normally.</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Wording</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Wording for the Universal Novice baseline.</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>UNV-NOV6; approved 2026-10-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CHG-UNV-016</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>catch-a-falling-friend</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Carry the Wounded</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>catch-a-falling-friend.md</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Tier / Type / Tags / Attribute</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Tier / minimum level: 1; Type: Skill / Utility; Tags: —; Attribute: Brawn</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Tier: Novice · Minimum level: 1; Type: Movement; Tags: Universal / Skill / Support; Attribute: Brawn</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Taxonomy</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Universal Novice standard: functional Type, Universal tag, Novice tier.</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>UNV-NOV7; approved 2026-10-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CHG-UNV-017</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>catch-a-falling-friend</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Carry the Wounded</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>catch-a-falling-friend.md</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Card text</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Reaction to catch a falling ally; situational.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Retitle Carry the Wounded; Brawn Maneuver to carry an adjacent willing or 0 HP creature at half Speed.</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Replacement</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Replacement for the Universal Novice baseline.</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>UNV-NOV7; approved 2026-10-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CHG-UNV-018</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>keep-your-bearings</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Keep Your Bearings</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>keep-your-bearings.md</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Tier / Type / Tags / Attribute</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Tier / minimum level: 1; Type: Skill / Utility; Tags: —; Attribute: Reason</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Tier: Novice · Minimum level: 1; Type: Utility; Tags: Universal / Skill / Exploration; Attribute: Reason</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Taxonomy</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Universal Novice standard: functional Type, Universal tag, Novice tier.</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>UNV-NOV8; approved 2026-10-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CHG-UNV-019</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>keep-your-bearings</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Keep Your Bearings</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>keep-your-bearings.md</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Card text</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Landmark detail check with 1/2/3 progress.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Navigation task progress: 1/2/3; simplified to the cumulative task mechanic.</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Mechanics</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Mechanics for the Universal Novice baseline.</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>UNV-NOV8; approved 2026-10-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CHG-UNV-020</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>notice-the-human-detail</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Read the Room</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>notice-the-human-detail.md</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Tier / Type / Tags / Attribute</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Tier / minimum level: 1; Type: Skill / Utility; Tags: —; Attribute: Reason</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Tier: Novice · Minimum level: 1; Type: Utility; Tags: Universal / Skill / Social / Investigation; Attribute: Reason</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Taxonomy</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Universal Novice standard: functional Type, Universal tag, Novice tier.</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>UNV-NOV9; approved 2026-10-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CHG-UNV-021</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>notice-the-human-detail</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Read the Room</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>notice-the-human-detail.md</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Card text</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>One-minute detail, inference and check.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Retitle Read the Room; investigation task progress: 1/2/3.</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Replacement</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Replacement for the Universal Novice baseline.</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>UNV-NOV9; approved 2026-10-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CHG-UNV-022</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>pack-with-purpose</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Pack with Purpose</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>pack-with-purpose.md</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Tier / Type / Tags / Attribute</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Tier / minimum level: 1; Type: Skill / Utility; Tags: —; Attribute: None — no roll</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Tier: Novice · Minimum level: 1; Type: Utility; Tags: Universal / Skill / Passive; Attribute: None (no roll)</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Taxonomy</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Universal Novice standard: functional Type, Universal tag, Novice tier.</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>UNV-NOV10; approved 2026-10-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CHG-UNV-023</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>pack-with-purpose</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Pack with Purpose</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>pack-with-purpose.md</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Card text</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Current text said it grants no free potion use or inventory benefit.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Positive wording; potions, inventory space and Bulk follow their normal rules.</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Wording</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Wording for the Universal Novice baseline.</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>UNV-NOV10; approved 2026-10-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CHG-UNV-024</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>tell-a-worthy-story</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Tell a Worthy Story</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>tell-a-worthy-story.md</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Tier / Type / Tags / Attribute</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Tier / minimum level: 1; Type: Skill / Utility; Tags: —; Attribute: Guile</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Tier: Novice · Minimum level: 1; Type: Utility; Tags: Universal / Skill / Social; Attribute: Guile</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Taxonomy</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Universal Novice standard: functional Type, Universal tag, Novice tier.</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>UNV-NOV11; approved 2026-10-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>CHG-UNV-025</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>tell-a-worthy-story</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Tell a Worthy Story</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>tell-a-worthy-story.md</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Card text</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Audience engagement with 1/2/3 progress.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Manipulation task progress: 1/2/3; tale-based persuasion or deception.</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Mechanics</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Mechanics for the Universal Novice baseline.</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>UNV-NOV11; approved 2026-10-29.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q204"/>

</xml_diff>

<commit_message>
Close Universal Novice at 13 of 13
Approves Conditioned Body Option C and Hold a Conversation with progress-only 2/3/4. Records CHG-UNV-026 through CHG-UNV-029.

Universal ladder review is complete: 13 Novice, 6 Adept, 3 Master. Book cards remain unchanged.
</commit_message>
<xml_diff>
--- a/review/abilities/workbooks/31_Novice_Abilities.xlsx
+++ b/review/abilities/workbooks/31_Novice_Abilities.xlsx
@@ -6718,19 +6718,17 @@
           <t>Level 1</t>
         </is>
       </c>
-      <c r="D55" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="D55" s="7" t="n">
+        <v>2</v>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>Training / Passive</t>
+          <t>Training</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Universal / Training / Passive</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
@@ -6740,12 +6738,12 @@
       </c>
       <c r="H55" s="7" t="inlineStr">
         <is>
-          <t>None — no roll</t>
+          <t>None (no roll)</t>
         </is>
       </c>
       <c r="I55" s="7" t="inlineStr">
         <is>
-          <t>Self</t>
+          <t>Self.</t>
         </is>
       </c>
       <c r="J55" s="7" t="inlineStr">
@@ -6760,17 +6758,17 @@
       </c>
       <c r="L55" s="7" t="inlineStr">
         <is>
-          <t>At most one purchase per level; unused purchases cannot be saved.</t>
+          <t>At most one purchase per level; each level's purchase stands on its own.</t>
         </is>
       </c>
       <c r="M55" s="7" t="inlineStr">
         <is>
-          <t>Increase maximum HP by 1.</t>
+          <t>Maximum HP +1 per purchase; once per level.</t>
         </is>
       </c>
       <c r="N55" s="7" t="inlineStr">
         <is>
-          <t>Maximum HP +1. At most one purchase at each level; missed purchases cannot be banked. No attribute increase.</t>
+          <t>Maximum HP +1 per purchase. Purchase once at each character level. Each level's purchase stands on its own. This ability increases maximum HP only.</t>
         </is>
       </c>
       <c r="O55" s="7" t="inlineStr">
@@ -6800,8 +6798,16 @@
 Assign a discipline requirement or formalize a General category.</t>
         </is>
       </c>
-      <c r="T55" s="7" t="inlineStr"/>
-      <c r="U55" s="7" t="inlineStr"/>
+      <c r="T55" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U55" s="7" t="inlineStr">
+        <is>
+          <t>UNV-NOV12; approved 2026-10-29. Option C; playtesting may revisit.</t>
+        </is>
+      </c>
       <c r="V55" s="7" t="inlineStr">
         <is>
           <t>conditioned-body.md</t>
@@ -6824,19 +6830,17 @@
           <t>Level 1</t>
         </is>
       </c>
-      <c r="D56" s="9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="D56" s="9" t="n">
+        <v>2</v>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Universal / Skill / Social</t>
         </is>
       </c>
       <c r="G56" s="9" t="inlineStr">
@@ -6851,12 +6855,12 @@
       </c>
       <c r="I56" s="9" t="inlineStr">
         <is>
-          <t>One nonhostile creature you share a language with; one minute</t>
+          <t>One nonhostile creature you share a language with.</t>
         </is>
       </c>
       <c r="J56" s="9" t="inlineStr">
         <is>
-          <t>Information and earned progress persist for the stated task; completed changes remain until circumstances alter them.</t>
+          <t>The progress persists for the social task.</t>
         </is>
       </c>
       <c r="K56" s="9" t="inlineStr">
@@ -6871,15 +6875,15 @@
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>Advance a conversation and learn concerns.</t>
+          <t>Make a Guile check for 2/3/4 progress toward a social task.</t>
         </is>
       </c>
       <c r="N56" s="9" t="inlineStr">
         <is>
-          <t>Expert social practice, not compulsory speech or a replacement for roleplay. No card is required to talk, persuade or ask questions.
-• Weak: 1 progress toward a plausible conversation objective; learn one topic the listener openly welcomes.
-• Standard: 2 progress; learn that topic and one concern the listener expresses about your request.
-• Strong: 3 progress, both details above, and a subject it openly shows reluctance to discuss.</t>
+          <t>Ordinary conversation remains available to everyone; this ability adds a reliable way to steer it. Choose one plausible conversation objective. Make a Guile check to make progress toward the social task.
+• Weak: 2 progress.
+• Standard: 3 progress.
+• Strong: 4 progress.</t>
         </is>
       </c>
       <c r="O56" s="9" t="inlineStr">
@@ -6907,8 +6911,16 @@
           <t>Assign a discipline requirement or formalize a General category.</t>
         </is>
       </c>
-      <c r="T56" s="9" t="inlineStr"/>
-      <c r="U56" s="9" t="inlineStr"/>
+      <c r="T56" s="9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U56" s="9" t="inlineStr">
+        <is>
+          <t>UNV-NOV13; approved 2026-10-29.</t>
+        </is>
+      </c>
       <c r="V56" s="9" t="inlineStr">
         <is>
           <t>hold-a-conversation.md</t>
@@ -20078,14 +20090,22 @@
           <t>None</t>
         </is>
       </c>
-      <c r="D55" s="7" t="inlineStr"/>
-      <c r="E55" s="7" t="inlineStr"/>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="n"/>
       <c r="F55" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G55" s="7" t="inlineStr"/>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
       <c r="H55" s="7" t="inlineStr">
         <is>
           <t>2</t>
@@ -20098,12 +20118,12 @@
       </c>
       <c r="J55" s="7" t="inlineStr">
         <is>
-          <t>Training / Passive</t>
+          <t>Training</t>
         </is>
       </c>
       <c r="K55" s="7" t="inlineStr">
         <is>
-          <t>No requirement; policy gap (F02).</t>
+          <t>No requirement; Universal (no discipline).</t>
         </is>
       </c>
     </row>
@@ -20123,14 +20143,22 @@
           <t>None</t>
         </is>
       </c>
-      <c r="D56" s="9" t="inlineStr"/>
-      <c r="E56" s="9" t="inlineStr"/>
+      <c r="D56" s="9" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="E56" s="9" t="n"/>
       <c r="F56" s="9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G56" s="9" t="inlineStr"/>
+      <c r="G56" s="9" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
       <c r="H56" s="9" t="inlineStr">
         <is>
           <t>2</t>
@@ -20143,12 +20171,12 @@
       </c>
       <c r="J56" s="9" t="inlineStr">
         <is>
-          <t>Skill / Utility</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="K56" s="9" t="inlineStr">
         <is>
-          <t>No requirement; policy gap (F02).</t>
+          <t>No requirement; Universal (no discipline).</t>
         </is>
       </c>
     </row>
@@ -25267,7 +25295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q29"/>
+  <dimension ref="A1:Q33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26458,7 +26486,6 @@
           <t>bruceamoser/heroes-of-legend-foundry#252</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
           <t>2026-10-29</t>
@@ -26541,7 +26568,6 @@
           <t>bruceamoser/heroes-of-legend-foundry#252</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
           <t>2026-10-29</t>
@@ -26624,7 +26650,6 @@
           <t>bruceamoser/heroes-of-legend-foundry#252</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
           <t>2026-10-29</t>
@@ -26707,7 +26732,6 @@
           <t>bruceamoser/heroes-of-legend-foundry#252</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
           <t>2026-10-29</t>
@@ -26790,7 +26814,6 @@
           <t>bruceamoser/heroes-of-legend-foundry#252</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
           <t>2026-10-29</t>
@@ -26873,7 +26896,6 @@
           <t>bruceamoser/heroes-of-legend-foundry#252</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
           <t>2026-10-29</t>
@@ -26956,7 +26978,6 @@
           <t>bruceamoser/heroes-of-legend-foundry#252</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
           <t>2026-10-29</t>
@@ -27039,7 +27060,6 @@
           <t>bruceamoser/heroes-of-legend-foundry#252</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
           <t>2026-10-29</t>
@@ -27122,7 +27142,6 @@
           <t>bruceamoser/heroes-of-legend-foundry#252</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
           <t>2026-10-29</t>
@@ -27205,7 +27224,6 @@
           <t>bruceamoser/heroes-of-legend-foundry#252</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
           <t>2026-10-29</t>
@@ -27288,7 +27306,6 @@
           <t>bruceamoser/heroes-of-legend-foundry#252</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
           <t>2026-10-29</t>
@@ -27371,7 +27388,6 @@
           <t>bruceamoser/heroes-of-legend-foundry#252</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
           <t>2026-10-29</t>
@@ -27454,7 +27470,6 @@
           <t>bruceamoser/heroes-of-legend-foundry#252</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
           <t>2026-10-29</t>
@@ -27463,6 +27478,336 @@
       <c r="Q29" t="inlineStr">
         <is>
           <t>UNV-NOV11; approved 2026-10-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>CHG-UNV-026</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>conditioned-body</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Conditioned Body</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>conditioned-body.md</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Tier / Type / Tags / Attribute</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Tier / minimum level: 1; Type: Training / Passive; Tags: —; Attribute: None — no roll</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Tier: Novice · Minimum level: 1; Type: Training; Tags: Universal / Training / Passive; Attribute: None (no roll)</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Taxonomy</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Universal Novice standard.</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>UNV-NOV12; approved 2026-10-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>CHG-UNV-027</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>conditioned-body</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Conditioned Body</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>conditioned-body.md</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Card text</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Maximum HP +1; at most one purchase at each level; missed purchases cannot be banked; no attribute increase.</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Maximum HP +1 per purchase; purchase once at each level; each level's purchase stands on its own; maximum HP only.</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Wording</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Option C confirmed; playtesting may revisit.</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>UNV-NOV12; approved 2026-10-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>CHG-UNV-028</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>hold-a-conversation</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Hold a Conversation</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>hold-a-conversation.md</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Tier / Type / Tags / Attribute</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Tier / minimum level: 1; Type: Skill / Utility; Tags: —; Attribute: Guile</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Tier: Novice · Minimum level: 1; Type: Utility; Tags: Universal / Skill / Social; Attribute: Guile</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Taxonomy</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Universal Novice standard.</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>UNV-NOV13; approved 2026-10-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>CHG-UNV-029</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>UNI-02</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>hold-a-conversation</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Hold a Conversation</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>hold-a-conversation.md</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Card text</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>1/2/3 progress plus topic, concern and reluctant subject; no compulsory speech or replacement for roleplay.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Progress only at 2/3/4; ordinary conversation remains available; one minute, Guile check, one social task.</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Mechanics</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Progress-only 2/3/4 approved.</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>UNV-NOV13; approved 2026-10-29.</t>
         </is>
       </c>
     </row>

</xml_diff>